<commit_message>
Show effort ratings as 'Effort to apply'
The tracker's How To Proceed column sometimes holds a bare effort rating
(MEDIUM, EASY) instead of instructions. Import now stores those as
Effort to apply; a one-time, idempotent migration moves existing imported
values out of Next action (logged per lead). Shown on the lead page and
as a column on the Ready list.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YKHGKKZo6qqGjZCvD1qCxQ
</commit_message>
<xml_diff>
--- a/tests/fixtures/sample-tracker.xlsx
+++ b/tests/fixtures/sample-tracker.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="170">
   <si>
     <t>Account</t>
   </si>
@@ -293,6 +293,9 @@
   </si>
   <si>
     <t>Placeholder brief</t>
+  </si>
+  <si>
+    <t>MEDIUM</t>
   </si>
   <si>
     <t>Ready to apply</t>
@@ -1227,28 +1230,31 @@
       <c r="R2" t="s">
         <v>91</v>
       </c>
+      <c r="T2" t="s">
+        <v>92</v>
+      </c>
       <c r="U2" t="s">
         <v>67</v>
       </c>
       <c r="V2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="X2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="U3" t="s">
         <v>67</v>
@@ -1276,10 +1282,10 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E1" t="s">
         <v>2</v>
@@ -1288,25 +1294,25 @@
         <v>75</v>
       </c>
       <c r="G1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J1" t="s">
         <v>80</v>
       </c>
       <c r="K1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="M1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="N1" t="s">
         <v>87</v>
@@ -1320,21 +1326,21 @@
         <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1345,10 +1351,10 @@
         <v>0</v>
       </c>
       <c r="C5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E5" t="s">
         <v>2</v>
@@ -1357,25 +1363,25 @@
         <v>75</v>
       </c>
       <c r="G5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J5" t="s">
         <v>80</v>
       </c>
       <c r="K5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="M5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="N5" t="s">
         <v>87</v>
@@ -1386,10 +1392,10 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -1411,13 +1417,13 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F1" t="s">
         <v>88</v>
@@ -1431,7 +1437,7 @@
         <v>58</v>
       </c>
       <c r="C2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D2" t="s">
         <v>59</v>
@@ -1440,7 +1446,7 @@
         <v>67</v>
       </c>
       <c r="F2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -1462,16 +1468,16 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1482,7 +1488,7 @@
         <v>52</v>
       </c>
       <c r="C2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D2" t="s">
         <v>53</v>
@@ -1491,7 +1497,7 @@
         <v>67</v>
       </c>
       <c r="F2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -1573,18 +1579,18 @@
         <v>88</v>
       </c>
       <c r="W1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="X1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="Y1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B2" t="s">
         <v>36</v>
@@ -1596,7 +1602,7 @@
         <v>38</v>
       </c>
       <c r="W2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="Y2" t="s">
         <v>67</v>
@@ -1604,7 +1610,7 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
@@ -1633,10 +1639,10 @@
         <v>76</v>
       </c>
       <c r="I5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K5" t="s">
         <v>85</v>
@@ -1645,42 +1651,42 @@
         <v>86</v>
       </c>
       <c r="M5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="O5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Q5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="R5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="S5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -1696,154 +1702,154 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B4" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B9" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B10" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B11" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B12" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B13" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>163</v>
+      </c>
+      <c r="B14" t="s">
         <v>162</v>
-      </c>
-      <c r="B14" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B15" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B16" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B17" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B18" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B19" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>